<commit_message>
Regenerar outputs con maestro actualizado (176 proyectos activos)
- maestro.proyectos.xlsx: versión actualizada del cliente (+3 proyectos)
- Consolidado_Carga_PM_Blend360.xlsx: recalculado con nueva cartera
- Informe_Carga_PMs_Blend360.docx: actualizado (Diana Rojas sube a 12 proyectos)
- Propuesta_Gestion_Asignacion_PM_Blend360.docx: actualizado
- Propuesta_Reasignacion_PM_Blend360_new.xlsx: nueva versión de propuesta
  (archivo original bloqueado por Excel al momento del commit; renombrar
  reemplazando Propuesta_Reasignacion_PM_Blend360.xlsx cuando se cierre)
- Gráficas actualizadas: proyectos activos, utilización, clientes apilado

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Asignación Proyectos/3. Output/Consolidado_Carga_PM_Blend360.xlsx
+++ b/Asignación Proyectos/3. Output/Consolidado_Carga_PM_Blend360.xlsx
@@ -859,7 +859,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>194</v>
@@ -1369,31 +1369,27 @@
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>Time Off &amp; Holiday</t>
-        </is>
-      </c>
-      <c r="C11" s="25" t="inlineStr">
-        <is>
-          <t>Vacaciones/Ausencia</t>
+          <t>INACTIVO SOC - IA Sociedades 2024-2025 - Fixed</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Facturable</t>
         </is>
       </c>
       <c r="D11" s="18" t="n">
         <v>9</v>
       </c>
       <c r="E11" s="18" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="F11" s="18" t="n">
-        <v>27</v>
+        <v>11</v>
       </c>
       <c r="G11" s="19" t="n">
         <v>0.04627249357326477</v>
       </c>
-      <c r="H11" s="16" t="inlineStr">
-        <is>
-          <t>Ausencia registrada</t>
-        </is>
-      </c>
+      <c r="H11" s="16" t="inlineStr"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="20" t="inlineStr">
@@ -1403,27 +1399,31 @@
       </c>
       <c r="B12" s="21" t="inlineStr">
         <is>
-          <t>INACTIVO SOC - IA Sociedades 2024-2025 - Fixed</t>
-        </is>
-      </c>
-      <c r="C12" s="17" t="inlineStr">
-        <is>
-          <t>Facturable</t>
+          <t>Time Off &amp; Holiday</t>
+        </is>
+      </c>
+      <c r="C12" s="25" t="inlineStr">
+        <is>
+          <t>Vacaciones/Ausencia</t>
         </is>
       </c>
       <c r="D12" s="22" t="n">
         <v>9</v>
       </c>
       <c r="E12" s="22" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F12" s="22" t="n">
-        <v>11</v>
+        <v>27</v>
       </c>
       <c r="G12" s="23" t="n">
         <v>0.04627249357326477</v>
       </c>
-      <c r="H12" s="21" t="inlineStr"/>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>Ausencia registrada</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="15" t="inlineStr">
@@ -2194,7 +2194,7 @@
       </c>
       <c r="B43" s="16" t="inlineStr">
         <is>
-          <t>UNA- OSE 61 Egresados -Fixed</t>
+          <t>UNA- OSE 61 Egresados - Ret</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
@@ -2206,10 +2206,10 @@
         <v>1</v>
       </c>
       <c r="E43" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="18" t="n">
         <v>1</v>
-      </c>
-      <c r="F43" s="18" t="n">
-        <v>2</v>
       </c>
       <c r="G43" s="19" t="n">
         <v>0.005154639175257731</v>
@@ -2224,7 +2224,7 @@
       </c>
       <c r="B44" s="21" t="inlineStr">
         <is>
-          <t>UNA- OSE 61 Egresados - Ret</t>
+          <t>UNA- OSE 61 Egresados -Fixed</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
@@ -2236,10 +2236,10 @@
         <v>1</v>
       </c>
       <c r="E44" s="22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F44" s="22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G44" s="23" t="n">
         <v>0.005154639175257731</v>
@@ -2422,7 +2422,7 @@
       </c>
       <c r="B54" s="21" t="inlineStr">
         <is>
-          <t>SAN - Soporte y mantenimiento Quipu 2025 - Ret</t>
+          <t>DIA - Aprovisionamiento multinube - Lote 3 - CLOUD</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
@@ -2434,10 +2434,10 @@
         <v>20</v>
       </c>
       <c r="E54" s="22" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F54" s="22" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G54" s="23" t="n">
         <v>0.1030927835051546</v>
@@ -2452,7 +2452,7 @@
       </c>
       <c r="B55" s="16" t="inlineStr">
         <is>
-          <t>DIA - Aprovisionamiento multinube - Lote 3 - CLOUD</t>
+          <t>SAN - Soporte y mantenimiento Quipu 2025 - Ret</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
@@ -2464,10 +2464,10 @@
         <v>20</v>
       </c>
       <c r="E55" s="18" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F55" s="18" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="G55" s="19" t="n">
         <v>0.1030927835051546</v>
@@ -3168,7 +3168,7 @@
       </c>
       <c r="B82" s="21" t="inlineStr">
         <is>
-          <t>CO - Superservicios renovacion observatorio de datos- Fixed</t>
+          <t>CO - Ministerio de educacion - Colombia Aprende Portal- Operation - Ret</t>
         </is>
       </c>
       <c r="C82" s="17" t="inlineStr">
@@ -3180,10 +3180,10 @@
         <v>17</v>
       </c>
       <c r="E82" s="22" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="F82" s="22" t="n">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="G82" s="23" t="n">
         <v>0.08762886597938144</v>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="B83" s="16" t="inlineStr">
         <is>
-          <t>CO - Ministerio de educacion - Colombia Aprende Portal- Operation - Ret</t>
+          <t>CO - Superservicios renovacion observatorio de datos- Fixed</t>
         </is>
       </c>
       <c r="C83" s="17" t="inlineStr">
@@ -3210,10 +3210,10 @@
         <v>17</v>
       </c>
       <c r="E83" s="18" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="F83" s="18" t="n">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="G83" s="19" t="n">
         <v>0.08762886597938144</v>
@@ -3883,7 +3883,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F169"/>
+  <dimension ref="A1:F172"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -5568,12 +5568,12 @@
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="15" t="inlineStr">
         <is>
-          <t>Indira Duarte</t>
+          <t>Diana Rojas</t>
         </is>
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>P2457</t>
+          <t>P2847</t>
         </is>
       </c>
       <c r="C55" s="15" t="inlineStr">
@@ -5583,12 +5583,12 @@
       </c>
       <c r="D55" s="16" t="inlineStr">
         <is>
-          <t>AI Auditoría Médica</t>
+          <t>peración Auditoria Cuentas Medicas</t>
         </is>
       </c>
       <c r="E55" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F55" s="16" t="inlineStr">
@@ -5600,12 +5600,12 @@
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="20" t="inlineStr">
         <is>
-          <t>Indira Duarte</t>
+          <t>Diana Rojas</t>
         </is>
       </c>
       <c r="B56" s="20" t="inlineStr">
         <is>
-          <t>P2470</t>
+          <t>P2848</t>
         </is>
       </c>
       <c r="C56" s="20" t="inlineStr">
@@ -5615,7 +5615,7 @@
       </c>
       <c r="D56" s="21" t="inlineStr">
         <is>
-          <t>AI Auditoría Médica</t>
+          <t>peración Auditoria Cuentas Medicas</t>
         </is>
       </c>
       <c r="E56" s="20" t="inlineStr">
@@ -5632,12 +5632,12 @@
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="15" t="inlineStr">
         <is>
-          <t>Indira Duarte</t>
+          <t>Diana Rojas</t>
         </is>
       </c>
       <c r="B57" s="15" t="inlineStr">
         <is>
-          <t>P2471</t>
+          <t>P2849</t>
         </is>
       </c>
       <c r="C57" s="15" t="inlineStr">
@@ -5647,7 +5647,7 @@
       </c>
       <c r="D57" s="16" t="inlineStr">
         <is>
-          <t>AI Auditoría Médica</t>
+          <t>peración Auditoria Cuentas Medicas</t>
         </is>
       </c>
       <c r="E57" s="15" t="inlineStr">
@@ -5669,7 +5669,7 @@
       </c>
       <c r="B58" s="20" t="inlineStr">
         <is>
-          <t>P2472</t>
+          <t>P2457</t>
         </is>
       </c>
       <c r="C58" s="20" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="E58" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F58" s="21" t="inlineStr">
@@ -5696,22 +5696,22 @@
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="15" t="inlineStr">
         <is>
-          <t>Juan Bernal</t>
+          <t>Indira Duarte</t>
         </is>
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>P1932</t>
+          <t>P2470</t>
         </is>
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>DIA</t>
+          <t>ADR</t>
         </is>
       </c>
       <c r="D59" s="16" t="inlineStr">
         <is>
-          <t>Aprovisionamiento multinube - Lote 3</t>
+          <t>AI Auditoría Médica</t>
         </is>
       </c>
       <c r="E59" s="15" t="inlineStr">
@@ -5721,71 +5721,71 @@
       </c>
       <c r="F59" s="16" t="inlineStr">
         <is>
-          <t>DIAN</t>
+          <t>La Administradora de los Recursos del Sistema General de Seguridad Social en Salud</t>
         </is>
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="20" t="inlineStr">
         <is>
-          <t>Juan Bernal</t>
+          <t>Indira Duarte</t>
         </is>
       </c>
       <c r="B60" s="20" t="inlineStr">
         <is>
-          <t>P2019</t>
+          <t>P2471</t>
         </is>
       </c>
       <c r="C60" s="20" t="inlineStr">
         <is>
-          <t>CJU</t>
+          <t>ADR</t>
         </is>
       </c>
       <c r="D60" s="21" t="inlineStr">
         <is>
-          <t>Vigilancia y MET Plus</t>
+          <t>AI Auditoría Médica</t>
         </is>
       </c>
       <c r="E60" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F60" s="21" t="inlineStr">
         <is>
-          <t>Coljuegos</t>
+          <t>La Administradora de los Recursos del Sistema General de Seguridad Social en Salud</t>
         </is>
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="15" t="inlineStr">
         <is>
-          <t>Juan Bernal</t>
+          <t>Indira Duarte</t>
         </is>
       </c>
       <c r="B61" s="15" t="inlineStr">
         <is>
-          <t>P2020</t>
+          <t>P2472</t>
         </is>
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>CJU</t>
+          <t>ADR</t>
         </is>
       </c>
       <c r="D61" s="16" t="inlineStr">
         <is>
-          <t>Vigilancia y MET Plus</t>
+          <t>AI Auditoría Médica</t>
         </is>
       </c>
       <c r="E61" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F61" s="16" t="inlineStr">
         <is>
-          <t>Coljuegos</t>
+          <t>La Administradora de los Recursos del Sistema General de Seguridad Social en Salud</t>
         </is>
       </c>
     </row>
@@ -5797,27 +5797,27 @@
       </c>
       <c r="B62" s="20" t="inlineStr">
         <is>
-          <t>P2021</t>
+          <t>P1932</t>
         </is>
       </c>
       <c r="C62" s="20" t="inlineStr">
         <is>
-          <t>CJU</t>
+          <t>DIA</t>
         </is>
       </c>
       <c r="D62" s="21" t="inlineStr">
         <is>
-          <t>Vigilancia y MET Plus</t>
+          <t>Aprovisionamiento multinube - Lote 3</t>
         </is>
       </c>
       <c r="E62" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F62" s="21" t="inlineStr">
         <is>
-          <t>Coljuegos</t>
+          <t>DIAN</t>
         </is>
       </c>
     </row>
@@ -5829,7 +5829,7 @@
       </c>
       <c r="B63" s="15" t="inlineStr">
         <is>
-          <t>P2022</t>
+          <t>P2019</t>
         </is>
       </c>
       <c r="C63" s="15" t="inlineStr">
@@ -5844,7 +5844,7 @@
       </c>
       <c r="E63" s="15" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F63" s="16" t="inlineStr">
@@ -5861,27 +5861,27 @@
       </c>
       <c r="B64" s="20" t="inlineStr">
         <is>
-          <t>P2240</t>
+          <t>P2020</t>
         </is>
       </c>
       <c r="C64" s="20" t="inlineStr">
         <is>
-          <t>ICF</t>
+          <t>CJU</t>
         </is>
       </c>
       <c r="D64" s="21" t="inlineStr">
         <is>
-          <t>Evolución Datalake Fase 2 2025</t>
+          <t>Vigilancia y MET Plus</t>
         </is>
       </c>
       <c r="E64" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F64" s="21" t="inlineStr">
         <is>
-          <t>Instituto Colombiano Para La Evaluacion De La Educacion ICFES</t>
+          <t>Coljuegos</t>
         </is>
       </c>
     </row>
@@ -5893,17 +5893,17 @@
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>P2559</t>
+          <t>P2021</t>
         </is>
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>ICF</t>
+          <t>CJU</t>
         </is>
       </c>
       <c r="D65" s="16" t="inlineStr">
         <is>
-          <t>Operacion en AWS</t>
+          <t>Vigilancia y MET Plus</t>
         </is>
       </c>
       <c r="E65" s="15" t="inlineStr">
@@ -5913,7 +5913,7 @@
       </c>
       <c r="F65" s="16" t="inlineStr">
         <is>
-          <t>ICFES</t>
+          <t>Coljuegos</t>
         </is>
       </c>
     </row>
@@ -5925,7 +5925,7 @@
       </c>
       <c r="B66" s="20" t="inlineStr">
         <is>
-          <t>P2615</t>
+          <t>P2022</t>
         </is>
       </c>
       <c r="C66" s="20" t="inlineStr">
@@ -5935,12 +5935,12 @@
       </c>
       <c r="D66" s="21" t="inlineStr">
         <is>
-          <t>CJU - Localizados</t>
+          <t>Vigilancia y MET Plus</t>
         </is>
       </c>
       <c r="E66" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F66" s="21" t="inlineStr">
@@ -5957,27 +5957,27 @@
       </c>
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>P2616</t>
+          <t>P2240</t>
         </is>
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>CJU</t>
+          <t>ICF</t>
         </is>
       </c>
       <c r="D67" s="16" t="inlineStr">
         <is>
-          <t>CJU - Localizados</t>
+          <t>Evolución Datalake Fase 2 2025</t>
         </is>
       </c>
       <c r="E67" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F67" s="16" t="inlineStr">
         <is>
-          <t>Coljuegos</t>
+          <t>Instituto Colombiano Para La Evaluacion De La Educacion ICFES</t>
         </is>
       </c>
     </row>
@@ -5989,17 +5989,17 @@
       </c>
       <c r="B68" s="20" t="inlineStr">
         <is>
-          <t>P2617</t>
+          <t>P2559</t>
         </is>
       </c>
       <c r="C68" s="20" t="inlineStr">
         <is>
-          <t>CJU</t>
+          <t>ICF</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
         <is>
-          <t>CJU - Localizados</t>
+          <t>Operacion en AWS</t>
         </is>
       </c>
       <c r="E68" s="20" t="inlineStr">
@@ -6009,7 +6009,7 @@
       </c>
       <c r="F68" s="21" t="inlineStr">
         <is>
-          <t>Coljuegos</t>
+          <t>ICFES</t>
         </is>
       </c>
     </row>
@@ -6021,7 +6021,7 @@
       </c>
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>P2618</t>
+          <t>P2615</t>
         </is>
       </c>
       <c r="C69" s="15" t="inlineStr">
@@ -6036,7 +6036,7 @@
       </c>
       <c r="E69" s="15" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F69" s="16" t="inlineStr">
@@ -6053,7 +6053,7 @@
       </c>
       <c r="B70" s="20" t="inlineStr">
         <is>
-          <t>P2619</t>
+          <t>P2616</t>
         </is>
       </c>
       <c r="C70" s="20" t="inlineStr">
@@ -6063,12 +6063,12 @@
       </c>
       <c r="D70" s="21" t="inlineStr">
         <is>
-          <t>CJU - STecnica</t>
+          <t>CJU - Localizados</t>
         </is>
       </c>
       <c r="E70" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F70" s="21" t="inlineStr">
@@ -6085,7 +6085,7 @@
       </c>
       <c r="B71" s="15" t="inlineStr">
         <is>
-          <t>P2620</t>
+          <t>P2617</t>
         </is>
       </c>
       <c r="C71" s="15" t="inlineStr">
@@ -6095,12 +6095,12 @@
       </c>
       <c r="D71" s="16" t="inlineStr">
         <is>
-          <t>CJU - STecnica</t>
+          <t>CJU - Localizados</t>
         </is>
       </c>
       <c r="E71" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F71" s="16" t="inlineStr">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="B72" s="20" t="inlineStr">
         <is>
-          <t>P2621</t>
+          <t>P2618</t>
         </is>
       </c>
       <c r="C72" s="20" t="inlineStr">
@@ -6127,12 +6127,12 @@
       </c>
       <c r="D72" s="21" t="inlineStr">
         <is>
-          <t>CJU - STecnica</t>
+          <t>CJU - Localizados</t>
         </is>
       </c>
       <c r="E72" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F72" s="21" t="inlineStr">
@@ -6149,7 +6149,7 @@
       </c>
       <c r="B73" s="15" t="inlineStr">
         <is>
-          <t>P2622</t>
+          <t>P2619</t>
         </is>
       </c>
       <c r="C73" s="15" t="inlineStr">
@@ -6164,7 +6164,7 @@
       </c>
       <c r="E73" s="15" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F73" s="16" t="inlineStr">
@@ -6181,27 +6181,27 @@
       </c>
       <c r="B74" s="20" t="inlineStr">
         <is>
-          <t>P2729</t>
+          <t>P2620</t>
         </is>
       </c>
       <c r="C74" s="20" t="inlineStr">
         <is>
-          <t>ICF</t>
+          <t>CJU</t>
         </is>
       </c>
       <c r="D74" s="21" t="inlineStr">
         <is>
-          <t>Banco de items Fase 2</t>
+          <t>CJU - STecnica</t>
         </is>
       </c>
       <c r="E74" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F74" s="21" t="inlineStr">
         <is>
-          <t>Icfes</t>
+          <t>Coljuegos</t>
         </is>
       </c>
     </row>
@@ -6213,17 +6213,17 @@
       </c>
       <c r="B75" s="15" t="inlineStr">
         <is>
-          <t>P2730</t>
+          <t>P2621</t>
         </is>
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>ICF</t>
+          <t>CJU</t>
         </is>
       </c>
       <c r="D75" s="16" t="inlineStr">
         <is>
-          <t>Banco de items Fase 2</t>
+          <t>CJU - STecnica</t>
         </is>
       </c>
       <c r="E75" s="15" t="inlineStr">
@@ -6233,7 +6233,7 @@
       </c>
       <c r="F75" s="16" t="inlineStr">
         <is>
-          <t>Icfes</t>
+          <t>Coljuegos</t>
         </is>
       </c>
     </row>
@@ -6245,27 +6245,27 @@
       </c>
       <c r="B76" s="20" t="inlineStr">
         <is>
-          <t>P2731</t>
+          <t>P2622</t>
         </is>
       </c>
       <c r="C76" s="20" t="inlineStr">
         <is>
-          <t>ICF</t>
+          <t>CJU</t>
         </is>
       </c>
       <c r="D76" s="21" t="inlineStr">
         <is>
-          <t>Banco de items Fase 2</t>
+          <t>CJU - STecnica</t>
         </is>
       </c>
       <c r="E76" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F76" s="21" t="inlineStr">
         <is>
-          <t>Icfes</t>
+          <t>Coljuegos</t>
         </is>
       </c>
     </row>
@@ -6277,7 +6277,7 @@
       </c>
       <c r="B77" s="15" t="inlineStr">
         <is>
-          <t>P2732</t>
+          <t>P2729</t>
         </is>
       </c>
       <c r="C77" s="15" t="inlineStr">
@@ -6287,7 +6287,7 @@
       </c>
       <c r="D77" s="16" t="inlineStr">
         <is>
-          <t>Datalake 2026-1</t>
+          <t>Banco de items Fase 2</t>
         </is>
       </c>
       <c r="E77" s="15" t="inlineStr">
@@ -6309,7 +6309,7 @@
       </c>
       <c r="B78" s="20" t="inlineStr">
         <is>
-          <t>P2733</t>
+          <t>P2730</t>
         </is>
       </c>
       <c r="C78" s="20" t="inlineStr">
@@ -6319,12 +6319,12 @@
       </c>
       <c r="D78" s="21" t="inlineStr">
         <is>
-          <t>Datalake 2026-1</t>
+          <t>Banco de items Fase 2</t>
         </is>
       </c>
       <c r="E78" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F78" s="21" t="inlineStr">
@@ -6341,7 +6341,7 @@
       </c>
       <c r="B79" s="15" t="inlineStr">
         <is>
-          <t>P2734</t>
+          <t>P2731</t>
         </is>
       </c>
       <c r="C79" s="15" t="inlineStr">
@@ -6351,12 +6351,12 @@
       </c>
       <c r="D79" s="16" t="inlineStr">
         <is>
-          <t>Datalake 2026-1</t>
+          <t>Banco de items Fase 2</t>
         </is>
       </c>
       <c r="E79" s="15" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F79" s="16" t="inlineStr">
@@ -6373,7 +6373,7 @@
       </c>
       <c r="B80" s="20" t="inlineStr">
         <is>
-          <t>P2742</t>
+          <t>P2732</t>
         </is>
       </c>
       <c r="C80" s="20" t="inlineStr">
@@ -6383,12 +6383,12 @@
       </c>
       <c r="D80" s="21" t="inlineStr">
         <is>
-          <t>Citación con Georreferenciación</t>
+          <t>Datalake 2026-1</t>
         </is>
       </c>
       <c r="E80" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F80" s="21" t="inlineStr">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="B81" s="15" t="inlineStr">
         <is>
-          <t>P2744</t>
+          <t>P2733</t>
         </is>
       </c>
       <c r="C81" s="15" t="inlineStr">
@@ -6415,12 +6415,12 @@
       </c>
       <c r="D81" s="16" t="inlineStr">
         <is>
-          <t>Citación con Georreferenciación</t>
+          <t>Datalake 2026-1</t>
         </is>
       </c>
       <c r="E81" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F81" s="16" t="inlineStr">
@@ -6437,7 +6437,7 @@
       </c>
       <c r="B82" s="20" t="inlineStr">
         <is>
-          <t>P2745</t>
+          <t>P2734</t>
         </is>
       </c>
       <c r="C82" s="20" t="inlineStr">
@@ -6447,7 +6447,7 @@
       </c>
       <c r="D82" s="21" t="inlineStr">
         <is>
-          <t>Citación con Georreferenciación</t>
+          <t>Datalake 2026-1</t>
         </is>
       </c>
       <c r="E82" s="20" t="inlineStr">
@@ -6469,7 +6469,7 @@
       </c>
       <c r="B83" s="15" t="inlineStr">
         <is>
-          <t>P2746</t>
+          <t>P2742</t>
         </is>
       </c>
       <c r="C83" s="15" t="inlineStr">
@@ -6484,7 +6484,7 @@
       </c>
       <c r="E83" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F83" s="16" t="inlineStr">
@@ -6501,7 +6501,7 @@
       </c>
       <c r="B84" s="20" t="inlineStr">
         <is>
-          <t>P2747</t>
+          <t>P2744</t>
         </is>
       </c>
       <c r="C84" s="20" t="inlineStr">
@@ -6516,7 +6516,7 @@
       </c>
       <c r="E84" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F84" s="21" t="inlineStr">
@@ -6528,96 +6528,96 @@
     <row r="85" ht="18" customHeight="1">
       <c r="A85" s="15" t="inlineStr">
         <is>
-          <t>Kelly Carbonell</t>
+          <t>Juan Bernal</t>
         </is>
       </c>
       <c r="B85" s="15" t="inlineStr">
         <is>
-          <t>P1923</t>
+          <t>P2745</t>
         </is>
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>CCC</t>
+          <t>ICF</t>
         </is>
       </c>
       <c r="D85" s="16" t="inlineStr">
         <is>
-          <t>IaaS para DRP</t>
+          <t>Citación con Georreferenciación</t>
         </is>
       </c>
       <c r="E85" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F85" s="16" t="inlineStr">
         <is>
-          <t>Cámara de Comercio de Cali</t>
+          <t>Icfes</t>
         </is>
       </c>
     </row>
     <row r="86" ht="18" customHeight="1">
       <c r="A86" s="20" t="inlineStr">
         <is>
-          <t>Kelly Carbonell</t>
+          <t>Juan Bernal</t>
         </is>
       </c>
       <c r="B86" s="20" t="inlineStr">
         <is>
-          <t>P2397</t>
+          <t>P2746</t>
         </is>
       </c>
       <c r="C86" s="20" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>ICF</t>
         </is>
       </c>
       <c r="D86" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Virtualización infraestructura Cali </t>
+          <t>Citación con Georreferenciación</t>
         </is>
       </c>
       <c r="E86" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F86" s="21" t="inlineStr">
         <is>
-          <t>Alcaldia de Cali</t>
+          <t>Icfes</t>
         </is>
       </c>
     </row>
     <row r="87" ht="18" customHeight="1">
       <c r="A87" s="15" t="inlineStr">
         <is>
-          <t>Kelly Carbonell</t>
+          <t>Juan Bernal</t>
         </is>
       </c>
       <c r="B87" s="15" t="inlineStr">
         <is>
-          <t>P2398</t>
+          <t>P2747</t>
         </is>
       </c>
       <c r="C87" s="15" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>ICF</t>
         </is>
       </c>
       <c r="D87" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Virtualización infraestructura Cali </t>
+          <t>Citación con Georreferenciación</t>
         </is>
       </c>
       <c r="E87" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F87" s="16" t="inlineStr">
         <is>
-          <t>Alcaldia de Cali</t>
+          <t>Icfes</t>
         </is>
       </c>
     </row>
@@ -6629,27 +6629,27 @@
       </c>
       <c r="B88" s="20" t="inlineStr">
         <is>
-          <t>P2399</t>
+          <t>P1923</t>
         </is>
       </c>
       <c r="C88" s="20" t="inlineStr">
         <is>
-          <t>ACA</t>
+          <t>CCC</t>
         </is>
       </c>
       <c r="D88" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Virtualización infraestructura Cali </t>
+          <t>IaaS para DRP</t>
         </is>
       </c>
       <c r="E88" s="20" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F88" s="21" t="inlineStr">
         <is>
-          <t>Alcaldia de Cali</t>
+          <t>Cámara de Comercio de Cali</t>
         </is>
       </c>
     </row>
@@ -6661,7 +6661,7 @@
       </c>
       <c r="B89" s="15" t="inlineStr">
         <is>
-          <t>P2400</t>
+          <t>P2397</t>
         </is>
       </c>
       <c r="C89" s="15" t="inlineStr">
@@ -6676,7 +6676,7 @@
       </c>
       <c r="E89" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F89" s="16" t="inlineStr">
@@ -6693,7 +6693,7 @@
       </c>
       <c r="B90" s="20" t="inlineStr">
         <is>
-          <t>P2404</t>
+          <t>P2398</t>
         </is>
       </c>
       <c r="C90" s="20" t="inlineStr">
@@ -6703,12 +6703,12 @@
       </c>
       <c r="D90" s="21" t="inlineStr">
         <is>
-          <t>Fase III DataCali</t>
+          <t xml:space="preserve"> Virtualización infraestructura Cali </t>
         </is>
       </c>
       <c r="E90" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F90" s="21" t="inlineStr">
@@ -6725,7 +6725,7 @@
       </c>
       <c r="B91" s="15" t="inlineStr">
         <is>
-          <t>P2405</t>
+          <t>P2399</t>
         </is>
       </c>
       <c r="C91" s="15" t="inlineStr">
@@ -6735,12 +6735,12 @@
       </c>
       <c r="D91" s="16" t="inlineStr">
         <is>
-          <t>Fase III DataCali</t>
+          <t xml:space="preserve"> Virtualización infraestructura Cali </t>
         </is>
       </c>
       <c r="E91" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F91" s="16" t="inlineStr">
@@ -6757,7 +6757,7 @@
       </c>
       <c r="B92" s="20" t="inlineStr">
         <is>
-          <t>P2541</t>
+          <t>P2400</t>
         </is>
       </c>
       <c r="C92" s="20" t="inlineStr">
@@ -6767,12 +6767,12 @@
       </c>
       <c r="D92" s="21" t="inlineStr">
         <is>
-          <t>Hacienda a un Click</t>
+          <t xml:space="preserve"> Virtualización infraestructura Cali </t>
         </is>
       </c>
       <c r="E92" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F92" s="21" t="inlineStr">
@@ -6789,7 +6789,7 @@
       </c>
       <c r="B93" s="15" t="inlineStr">
         <is>
-          <t>P2542</t>
+          <t>P2404</t>
         </is>
       </c>
       <c r="C93" s="15" t="inlineStr">
@@ -6799,12 +6799,12 @@
       </c>
       <c r="D93" s="16" t="inlineStr">
         <is>
-          <t>Hacienda a un Click</t>
+          <t>Fase III DataCali</t>
         </is>
       </c>
       <c r="E93" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F93" s="16" t="inlineStr">
@@ -6821,7 +6821,7 @@
       </c>
       <c r="B94" s="20" t="inlineStr">
         <is>
-          <t>P2543</t>
+          <t>P2405</t>
         </is>
       </c>
       <c r="C94" s="20" t="inlineStr">
@@ -6831,12 +6831,12 @@
       </c>
       <c r="D94" s="21" t="inlineStr">
         <is>
-          <t>Hacienda a un Click</t>
+          <t>Fase III DataCali</t>
         </is>
       </c>
       <c r="E94" s="20" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F94" s="21" t="inlineStr">
@@ -6853,7 +6853,7 @@
       </c>
       <c r="B95" s="15" t="inlineStr">
         <is>
-          <t>P2544</t>
+          <t>P2541</t>
         </is>
       </c>
       <c r="C95" s="15" t="inlineStr">
@@ -6868,7 +6868,7 @@
       </c>
       <c r="E95" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F95" s="16" t="inlineStr">
@@ -6885,7 +6885,7 @@
       </c>
       <c r="B96" s="20" t="inlineStr">
         <is>
-          <t>P2822</t>
+          <t>P2542</t>
         </is>
       </c>
       <c r="C96" s="20" t="inlineStr">
@@ -6895,12 +6895,12 @@
       </c>
       <c r="D96" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secretaría de Transparencia MVP </t>
+          <t>Hacienda a un Click</t>
         </is>
       </c>
       <c r="E96" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F96" s="21" t="inlineStr">
@@ -6917,7 +6917,7 @@
       </c>
       <c r="B97" s="15" t="inlineStr">
         <is>
-          <t>P2823</t>
+          <t>P2543</t>
         </is>
       </c>
       <c r="C97" s="15" t="inlineStr">
@@ -6927,12 +6927,12 @@
       </c>
       <c r="D97" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secretaría de Transparencia MVP </t>
+          <t>Hacienda a un Click</t>
         </is>
       </c>
       <c r="E97" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F97" s="16" t="inlineStr">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="B98" s="20" t="inlineStr">
         <is>
-          <t>P2824</t>
+          <t>P2544</t>
         </is>
       </c>
       <c r="C98" s="20" t="inlineStr">
@@ -6959,12 +6959,12 @@
       </c>
       <c r="D98" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Secretaría de Transparencia MVP </t>
+          <t>Hacienda a un Click</t>
         </is>
       </c>
       <c r="E98" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F98" s="21" t="inlineStr">
@@ -6976,96 +6976,96 @@
     <row r="99" ht="18" customHeight="1">
       <c r="A99" s="15" t="inlineStr">
         <is>
-          <t>Miguel Garcia</t>
+          <t>Kelly Carbonell</t>
         </is>
       </c>
       <c r="B99" s="15" t="inlineStr">
         <is>
-          <t>P1966</t>
+          <t>P2822</t>
         </is>
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
-          <t>SPD</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="D99" s="16" t="inlineStr">
         <is>
-          <t>Repositorio Único de Datos</t>
+          <t xml:space="preserve">Secretaría de Transparencia MVP </t>
         </is>
       </c>
       <c r="E99" s="15" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F99" s="16" t="inlineStr">
         <is>
-          <t>Superintendencia Servicios Públicos Domiciliarios</t>
+          <t>Alcaldia de Cali</t>
         </is>
       </c>
     </row>
     <row r="100" ht="18" customHeight="1">
       <c r="A100" s="20" t="inlineStr">
         <is>
-          <t>Miguel Garcia</t>
+          <t>Kelly Carbonell</t>
         </is>
       </c>
       <c r="B100" s="20" t="inlineStr">
         <is>
-          <t>P1967</t>
+          <t>P2823</t>
         </is>
       </c>
       <c r="C100" s="20" t="inlineStr">
         <is>
-          <t>SPD</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="D100" s="21" t="inlineStr">
         <is>
-          <t>Repositorio Único de Datos</t>
+          <t xml:space="preserve">Secretaría de Transparencia MVP </t>
         </is>
       </c>
       <c r="E100" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F100" s="21" t="inlineStr">
         <is>
-          <t>Superintendencia Servicios Públicos Domiciliarios</t>
+          <t>Alcaldia de Cali</t>
         </is>
       </c>
     </row>
     <row r="101" ht="18" customHeight="1">
       <c r="A101" s="15" t="inlineStr">
         <is>
-          <t>Miguel Garcia</t>
+          <t>Kelly Carbonell</t>
         </is>
       </c>
       <c r="B101" s="15" t="inlineStr">
         <is>
-          <t>P2431</t>
+          <t>P2824</t>
         </is>
       </c>
       <c r="C101" s="15" t="inlineStr">
         <is>
-          <t>SED</t>
+          <t>ACA</t>
         </is>
       </c>
       <c r="D101" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automatización procesos seguros, adquisiciones y accidentes </t>
+          <t xml:space="preserve">Secretaría de Transparencia MVP </t>
         </is>
       </c>
       <c r="E101" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F101" s="16" t="inlineStr">
         <is>
-          <t>Secretaría de Educación del Distrito</t>
+          <t>Alcaldia de Cali</t>
         </is>
       </c>
     </row>
@@ -7077,17 +7077,17 @@
       </c>
       <c r="B102" s="20" t="inlineStr">
         <is>
-          <t>P2561</t>
+          <t>P1966</t>
         </is>
       </c>
       <c r="C102" s="20" t="inlineStr">
         <is>
-          <t>SED</t>
+          <t>SPD</t>
         </is>
       </c>
       <c r="D102" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automatización procesos seguros, adquisiciones y accidentes </t>
+          <t>Repositorio Único de Datos</t>
         </is>
       </c>
       <c r="E102" s="20" t="inlineStr">
@@ -7097,7 +7097,7 @@
       </c>
       <c r="F102" s="21" t="inlineStr">
         <is>
-          <t>Secretaría de Educación del Distrito</t>
+          <t>Superintendencia Servicios Públicos Domiciliarios</t>
         </is>
       </c>
     </row>
@@ -7109,27 +7109,27 @@
       </c>
       <c r="B103" s="15" t="inlineStr">
         <is>
-          <t>P2562</t>
+          <t>P1967</t>
         </is>
       </c>
       <c r="C103" s="15" t="inlineStr">
         <is>
-          <t>SED</t>
+          <t>SPD</t>
         </is>
       </c>
       <c r="D103" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Automatización procesos seguros, adquisiciones y accidentes </t>
+          <t>Repositorio Único de Datos</t>
         </is>
       </c>
       <c r="E103" s="15" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F103" s="16" t="inlineStr">
         <is>
-          <t>Secretaría de Educación del Distrito</t>
+          <t>Superintendencia Servicios Públicos Domiciliarios</t>
         </is>
       </c>
     </row>
@@ -7141,7 +7141,7 @@
       </c>
       <c r="B104" s="20" t="inlineStr">
         <is>
-          <t>P2563</t>
+          <t>P2431</t>
         </is>
       </c>
       <c r="C104" s="20" t="inlineStr">
@@ -7156,7 +7156,7 @@
       </c>
       <c r="E104" s="20" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F104" s="21" t="inlineStr">
@@ -7173,27 +7173,27 @@
       </c>
       <c r="B105" s="15" t="inlineStr">
         <is>
-          <t>P2611</t>
+          <t>P2561</t>
         </is>
       </c>
       <c r="C105" s="15" t="inlineStr">
         <is>
-          <t>MEN</t>
+          <t>SED</t>
         </is>
       </c>
       <c r="D105" s="16" t="inlineStr">
         <is>
-          <t>Operacion en AWS</t>
+          <t xml:space="preserve">Automatización procesos seguros, adquisiciones y accidentes </t>
         </is>
       </c>
       <c r="E105" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F105" s="16" t="inlineStr">
         <is>
-          <t>Ministerio de educación Nacional</t>
+          <t>Secretaría de Educación del Distrito</t>
         </is>
       </c>
     </row>
@@ -7205,27 +7205,27 @@
       </c>
       <c r="B106" s="20" t="inlineStr">
         <is>
-          <t>P2612</t>
+          <t>P2562</t>
         </is>
       </c>
       <c r="C106" s="20" t="inlineStr">
         <is>
-          <t>MEN</t>
+          <t>SED</t>
         </is>
       </c>
       <c r="D106" s="21" t="inlineStr">
         <is>
-          <t>Operacion en AWS</t>
+          <t xml:space="preserve">Automatización procesos seguros, adquisiciones y accidentes </t>
         </is>
       </c>
       <c r="E106" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F106" s="21" t="inlineStr">
         <is>
-          <t>Ministerio de educación Nacional</t>
+          <t>Secretaría de Educación del Distrito</t>
         </is>
       </c>
     </row>
@@ -7237,27 +7237,27 @@
       </c>
       <c r="B107" s="15" t="inlineStr">
         <is>
-          <t>P2634</t>
+          <t>P2563</t>
         </is>
       </c>
       <c r="C107" s="15" t="inlineStr">
         <is>
-          <t>MEN</t>
+          <t>SED</t>
         </is>
       </c>
       <c r="D107" s="16" t="inlineStr">
         <is>
-          <t>Operacion en AWS</t>
+          <t xml:space="preserve">Automatización procesos seguros, adquisiciones y accidentes </t>
         </is>
       </c>
       <c r="E107" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F107" s="16" t="inlineStr">
         <is>
-          <t>Ministerio de educación Nacional</t>
+          <t>Secretaría de Educación del Distrito</t>
         </is>
       </c>
     </row>
@@ -7269,17 +7269,17 @@
       </c>
       <c r="B108" s="20" t="inlineStr">
         <is>
-          <t>P2671</t>
+          <t>P2611</t>
         </is>
       </c>
       <c r="C108" s="20" t="inlineStr">
         <is>
-          <t>HPL</t>
+          <t>MEN</t>
         </is>
       </c>
       <c r="D108" s="21" t="inlineStr">
         <is>
-          <t>AWS Database Migration &amp; Modernization</t>
+          <t>Operacion en AWS</t>
         </is>
       </c>
       <c r="E108" s="20" t="inlineStr">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="F108" s="21" t="inlineStr">
         <is>
-          <t xml:space="preserve">HotelPlanner </t>
+          <t>Ministerio de educación Nacional</t>
         </is>
       </c>
     </row>
@@ -7301,27 +7301,27 @@
       </c>
       <c r="B109" s="15" t="inlineStr">
         <is>
-          <t>P2723</t>
+          <t>P2612</t>
         </is>
       </c>
       <c r="C109" s="15" t="inlineStr">
         <is>
-          <t>SPD</t>
+          <t>MEN</t>
         </is>
       </c>
       <c r="D109" s="16" t="inlineStr">
         <is>
-          <t>Renovacion observatorio de datos-</t>
+          <t>Operacion en AWS</t>
         </is>
       </c>
       <c r="E109" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F109" s="16" t="inlineStr">
         <is>
-          <t>Superintendencia Servicios Públicos Domiciliarios</t>
+          <t>Ministerio de educación Nacional</t>
         </is>
       </c>
     </row>
@@ -7333,27 +7333,27 @@
       </c>
       <c r="B110" s="20" t="inlineStr">
         <is>
-          <t>P2724</t>
+          <t>P2634</t>
         </is>
       </c>
       <c r="C110" s="20" t="inlineStr">
         <is>
-          <t>SPD</t>
+          <t>MEN</t>
         </is>
       </c>
       <c r="D110" s="21" t="inlineStr">
         <is>
-          <t>Renovacion observatorio de datos-</t>
+          <t>Operacion en AWS</t>
         </is>
       </c>
       <c r="E110" s="20" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F110" s="21" t="inlineStr">
         <is>
-          <t>Superintendencia Servicios Públicos Domiciliarios</t>
+          <t>Ministerio de educación Nacional</t>
         </is>
       </c>
     </row>
@@ -7365,27 +7365,27 @@
       </c>
       <c r="B111" s="15" t="inlineStr">
         <is>
-          <t>P2725</t>
+          <t>P2671</t>
         </is>
       </c>
       <c r="C111" s="15" t="inlineStr">
         <is>
-          <t>SPD</t>
+          <t>HPL</t>
         </is>
       </c>
       <c r="D111" s="16" t="inlineStr">
         <is>
-          <t>Renovacion observatorio de datos-</t>
+          <t>AWS Database Migration &amp; Modernization</t>
         </is>
       </c>
       <c r="E111" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F111" s="16" t="inlineStr">
         <is>
-          <t>Superintendencia Servicios Públicos Domiciliarios</t>
+          <t xml:space="preserve">HotelPlanner </t>
         </is>
       </c>
     </row>
@@ -7397,27 +7397,27 @@
       </c>
       <c r="B112" s="20" t="inlineStr">
         <is>
-          <t>P2726</t>
+          <t>P2786</t>
         </is>
       </c>
       <c r="C112" s="20" t="inlineStr">
         <is>
-          <t>SPD</t>
+          <t>HPL</t>
         </is>
       </c>
       <c r="D112" s="21" t="inlineStr">
         <is>
-          <t>Renovacion observatorio de datos-</t>
+          <t>AWS Database Migration &amp; Modernization</t>
         </is>
       </c>
       <c r="E112" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F112" s="21" t="inlineStr">
         <is>
-          <t>Superintendencia Servicios Públicos Domiciliarios</t>
+          <t xml:space="preserve">HotelPlanner </t>
         </is>
       </c>
     </row>
@@ -7429,49 +7429,49 @@
       </c>
       <c r="B113" s="15" t="inlineStr">
         <is>
-          <t>P2786</t>
+          <t>P2723</t>
         </is>
       </c>
       <c r="C113" s="15" t="inlineStr">
         <is>
-          <t>HPL</t>
+          <t>SPD</t>
         </is>
       </c>
       <c r="D113" s="16" t="inlineStr">
         <is>
-          <t>AWS Database Migration &amp; Modernization</t>
+          <t>Renovacion observatorio de datos-</t>
         </is>
       </c>
       <c r="E113" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F113" s="16" t="inlineStr">
         <is>
-          <t xml:space="preserve">HotelPlanner </t>
+          <t>Superintendencia Servicios Públicos Domiciliarios</t>
         </is>
       </c>
     </row>
     <row r="114" ht="18" customHeight="1">
       <c r="A114" s="20" t="inlineStr">
         <is>
-          <t>Oscar Barragan</t>
+          <t>Miguel Garcia</t>
         </is>
       </c>
       <c r="B114" s="20" t="inlineStr">
         <is>
-          <t>P1920</t>
+          <t>P2724</t>
         </is>
       </c>
       <c r="C114" s="20" t="inlineStr">
         <is>
-          <t>BTG</t>
+          <t>SPD</t>
         </is>
       </c>
       <c r="D114" s="21" t="inlineStr">
         <is>
-          <t>SmartCash - Operación</t>
+          <t>Renovacion observatorio de datos-</t>
         </is>
       </c>
       <c r="E114" s="20" t="inlineStr">
@@ -7481,61 +7481,61 @@
       </c>
       <c r="F114" s="21" t="inlineStr">
         <is>
-          <t>BTG Pactual Colombia</t>
+          <t>Superintendencia Servicios Públicos Domiciliarios</t>
         </is>
       </c>
     </row>
     <row r="115" ht="18" customHeight="1">
       <c r="A115" s="15" t="inlineStr">
         <is>
-          <t>Oscar Barragan</t>
+          <t>Miguel Garcia</t>
         </is>
       </c>
       <c r="B115" s="15" t="inlineStr">
         <is>
-          <t>P2012</t>
+          <t>P2725</t>
         </is>
       </c>
       <c r="C115" s="15" t="inlineStr">
         <is>
-          <t>BTG</t>
+          <t>SPD</t>
         </is>
       </c>
       <c r="D115" s="16" t="inlineStr">
         <is>
-          <t>SmartCash - Operación</t>
+          <t>Renovacion observatorio de datos-</t>
         </is>
       </c>
       <c r="E115" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F115" s="16" t="inlineStr">
         <is>
-          <t>BTG Pactual</t>
+          <t>Superintendencia Servicios Públicos Domiciliarios</t>
         </is>
       </c>
     </row>
     <row r="116" ht="18" customHeight="1">
       <c r="A116" s="20" t="inlineStr">
         <is>
-          <t>Oscar Barragan</t>
+          <t>Miguel Garcia</t>
         </is>
       </c>
       <c r="B116" s="20" t="inlineStr">
         <is>
-          <t>P1991</t>
+          <t>P2726</t>
         </is>
       </c>
       <c r="C116" s="20" t="inlineStr">
         <is>
-          <t>UNA</t>
+          <t>SPD</t>
         </is>
       </c>
       <c r="D116" s="21" t="inlineStr">
         <is>
-          <t>Unisalud</t>
+          <t>Renovacion observatorio de datos-</t>
         </is>
       </c>
       <c r="E116" s="20" t="inlineStr">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="F116" s="21" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Colombia</t>
+          <t>Superintendencia Servicios Públicos Domiciliarios</t>
         </is>
       </c>
     </row>
@@ -7557,27 +7557,27 @@
       </c>
       <c r="B117" s="15" t="inlineStr">
         <is>
-          <t>P1994</t>
+          <t>P1920</t>
         </is>
       </c>
       <c r="C117" s="15" t="inlineStr">
         <is>
-          <t>UNA</t>
+          <t>BTG</t>
         </is>
       </c>
       <c r="D117" s="16" t="inlineStr">
         <is>
-          <t>Regalías Sikie</t>
+          <t>SmartCash - Operación</t>
         </is>
       </c>
       <c r="E117" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F117" s="16" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Colombia</t>
+          <t>BTG Pactual Colombia</t>
         </is>
       </c>
     </row>
@@ -7589,17 +7589,17 @@
       </c>
       <c r="B118" s="20" t="inlineStr">
         <is>
-          <t>P2537</t>
+          <t>P2012</t>
         </is>
       </c>
       <c r="C118" s="20" t="inlineStr">
         <is>
-          <t>UNA</t>
+          <t>BTG</t>
         </is>
       </c>
       <c r="D118" s="21" t="inlineStr">
         <is>
-          <t>Regalías Sikie</t>
+          <t>SmartCash - Operación</t>
         </is>
       </c>
       <c r="E118" s="20" t="inlineStr">
@@ -7609,7 +7609,7 @@
       </c>
       <c r="F118" s="21" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Colombia</t>
+          <t>BTG Pactual</t>
         </is>
       </c>
     </row>
@@ -7621,7 +7621,7 @@
       </c>
       <c r="B119" s="15" t="inlineStr">
         <is>
-          <t>P2537</t>
+          <t>P1991</t>
         </is>
       </c>
       <c r="C119" s="15" t="inlineStr">
@@ -7631,7 +7631,7 @@
       </c>
       <c r="D119" s="16" t="inlineStr">
         <is>
-          <t>Regalías Sikie</t>
+          <t>Unisalud</t>
         </is>
       </c>
       <c r="E119" s="15" t="inlineStr">
@@ -7653,7 +7653,7 @@
       </c>
       <c r="B120" s="20" t="inlineStr">
         <is>
-          <t>P1977</t>
+          <t>P1994</t>
         </is>
       </c>
       <c r="C120" s="20" t="inlineStr">
@@ -7663,12 +7663,12 @@
       </c>
       <c r="D120" s="21" t="inlineStr">
         <is>
-          <t>Fortinet</t>
+          <t>Regalías Sikie</t>
         </is>
       </c>
       <c r="E120" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F120" s="21" t="inlineStr">
@@ -7685,7 +7685,7 @@
       </c>
       <c r="B121" s="15" t="inlineStr">
         <is>
-          <t>P1978</t>
+          <t>P2537</t>
         </is>
       </c>
       <c r="C121" s="15" t="inlineStr">
@@ -7695,12 +7695,12 @@
       </c>
       <c r="D121" s="16" t="inlineStr">
         <is>
-          <t>Fortinet</t>
+          <t>Regalías Sikie</t>
         </is>
       </c>
       <c r="E121" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F121" s="16" t="inlineStr">
@@ -7717,7 +7717,7 @@
       </c>
       <c r="B122" s="20" t="inlineStr">
         <is>
-          <t>P1983</t>
+          <t>P2537</t>
         </is>
       </c>
       <c r="C122" s="20" t="inlineStr">
@@ -7727,12 +7727,12 @@
       </c>
       <c r="D122" s="21" t="inlineStr">
         <is>
-          <t>Laboratorios Virtuales</t>
+          <t>Regalías Sikie</t>
         </is>
       </c>
       <c r="E122" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F122" s="21" t="inlineStr">
@@ -7749,7 +7749,7 @@
       </c>
       <c r="B123" s="15" t="inlineStr">
         <is>
-          <t>P1973</t>
+          <t>P1977</t>
         </is>
       </c>
       <c r="C123" s="15" t="inlineStr">
@@ -7759,12 +7759,12 @@
       </c>
       <c r="D123" s="16" t="inlineStr">
         <is>
-          <t>Editorial de UNAL</t>
+          <t>Fortinet</t>
         </is>
       </c>
       <c r="E123" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F123" s="16" t="inlineStr">
@@ -7781,7 +7781,7 @@
       </c>
       <c r="B124" s="20" t="inlineStr">
         <is>
-          <t>P1988</t>
+          <t>P1978</t>
         </is>
       </c>
       <c r="C124" s="20" t="inlineStr">
@@ -7791,7 +7791,7 @@
       </c>
       <c r="D124" s="21" t="inlineStr">
         <is>
-          <t>Repositorio</t>
+          <t>Fortinet</t>
         </is>
       </c>
       <c r="E124" s="20" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="B125" s="15" t="inlineStr">
         <is>
-          <t>P1982</t>
+          <t>P1983</t>
         </is>
       </c>
       <c r="C125" s="15" t="inlineStr">
@@ -7823,7 +7823,7 @@
       </c>
       <c r="D125" s="16" t="inlineStr">
         <is>
-          <t>HPC Registro y Matrícula</t>
+          <t>Laboratorios Virtuales</t>
         </is>
       </c>
       <c r="E125" s="15" t="inlineStr">
@@ -7845,7 +7845,7 @@
       </c>
       <c r="B126" s="20" t="inlineStr">
         <is>
-          <t>P1979</t>
+          <t>P1973</t>
         </is>
       </c>
       <c r="C126" s="20" t="inlineStr">
@@ -7855,12 +7855,12 @@
       </c>
       <c r="D126" s="21" t="inlineStr">
         <is>
-          <t>Gestión de Información</t>
+          <t>Editorial de UNAL</t>
         </is>
       </c>
       <c r="E126" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F126" s="21" t="inlineStr">
@@ -7877,7 +7877,7 @@
       </c>
       <c r="B127" s="15" t="inlineStr">
         <is>
-          <t>P1980</t>
+          <t>P1988</t>
         </is>
       </c>
       <c r="C127" s="15" t="inlineStr">
@@ -7887,12 +7887,12 @@
       </c>
       <c r="D127" s="16" t="inlineStr">
         <is>
-          <t>Gestión de Información</t>
+          <t>Repositorio</t>
         </is>
       </c>
       <c r="E127" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F127" s="16" t="inlineStr">
@@ -7909,7 +7909,7 @@
       </c>
       <c r="B128" s="20" t="inlineStr">
         <is>
-          <t>P1981</t>
+          <t>P1982</t>
         </is>
       </c>
       <c r="C128" s="20" t="inlineStr">
@@ -7919,7 +7919,7 @@
       </c>
       <c r="D128" s="21" t="inlineStr">
         <is>
-          <t>Gestión de Información</t>
+          <t>HPC Registro y Matrícula</t>
         </is>
       </c>
       <c r="E128" s="20" t="inlineStr">
@@ -7941,7 +7941,7 @@
       </c>
       <c r="B129" s="15" t="inlineStr">
         <is>
-          <t>P1975</t>
+          <t>P1979</t>
         </is>
       </c>
       <c r="C129" s="15" t="inlineStr">
@@ -7951,12 +7951,12 @@
       </c>
       <c r="D129" s="16" t="inlineStr">
         <is>
-          <t>Facultad de ingenieria</t>
+          <t>Gestión de Información</t>
         </is>
       </c>
       <c r="E129" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F129" s="16" t="inlineStr">
@@ -7973,7 +7973,7 @@
       </c>
       <c r="B130" s="20" t="inlineStr">
         <is>
-          <t>P2036</t>
+          <t>P1980</t>
         </is>
       </c>
       <c r="C130" s="20" t="inlineStr">
@@ -7983,12 +7983,12 @@
       </c>
       <c r="D130" s="21" t="inlineStr">
         <is>
-          <t>Facultad de ingenieria</t>
+          <t>Gestión de Información</t>
         </is>
       </c>
       <c r="E130" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F130" s="21" t="inlineStr">
@@ -8005,7 +8005,7 @@
       </c>
       <c r="B131" s="15" t="inlineStr">
         <is>
-          <t>P1990</t>
+          <t>P1981</t>
         </is>
       </c>
       <c r="C131" s="15" t="inlineStr">
@@ -8015,12 +8015,12 @@
       </c>
       <c r="D131" s="16" t="inlineStr">
         <is>
-          <t>Soporte y Mtto Quipu 2025</t>
+          <t>Gestión de Información</t>
         </is>
       </c>
       <c r="E131" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F131" s="16" t="inlineStr">
@@ -8037,7 +8037,7 @@
       </c>
       <c r="B132" s="20" t="inlineStr">
         <is>
-          <t>P2037</t>
+          <t>P1975</t>
         </is>
       </c>
       <c r="C132" s="20" t="inlineStr">
@@ -8047,12 +8047,12 @@
       </c>
       <c r="D132" s="21" t="inlineStr">
         <is>
-          <t>Facultad de Derecho concurso méritos</t>
+          <t>Facultad de ingenieria</t>
         </is>
       </c>
       <c r="E132" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F132" s="21" t="inlineStr">
@@ -8069,7 +8069,7 @@
       </c>
       <c r="B133" s="15" t="inlineStr">
         <is>
-          <t>P2038</t>
+          <t>P2036</t>
         </is>
       </c>
       <c r="C133" s="15" t="inlineStr">
@@ -8079,12 +8079,12 @@
       </c>
       <c r="D133" s="16" t="inlineStr">
         <is>
-          <t>Facultad de Derecho concurso méritos</t>
+          <t>Facultad de ingenieria</t>
         </is>
       </c>
       <c r="E133" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F133" s="16" t="inlineStr">
@@ -8101,7 +8101,7 @@
       </c>
       <c r="B134" s="20" t="inlineStr">
         <is>
-          <t>P2066</t>
+          <t>P1990</t>
         </is>
       </c>
       <c r="C134" s="20" t="inlineStr">
@@ -8111,12 +8111,12 @@
       </c>
       <c r="D134" s="21" t="inlineStr">
         <is>
-          <t>OSE 26 Admisiones</t>
+          <t>Soporte y Mtto Quipu 2025</t>
         </is>
       </c>
       <c r="E134" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F134" s="21" t="inlineStr">
@@ -8133,7 +8133,7 @@
       </c>
       <c r="B135" s="15" t="inlineStr">
         <is>
-          <t>P2067</t>
+          <t>P2037</t>
         </is>
       </c>
       <c r="C135" s="15" t="inlineStr">
@@ -8143,7 +8143,7 @@
       </c>
       <c r="D135" s="16" t="inlineStr">
         <is>
-          <t>OSE 43 Moodle Extensión</t>
+          <t>Facultad de Derecho concurso méritos</t>
         </is>
       </c>
       <c r="E135" s="15" t="inlineStr">
@@ -8165,7 +8165,7 @@
       </c>
       <c r="B136" s="20" t="inlineStr">
         <is>
-          <t>P2560</t>
+          <t>P2038</t>
         </is>
       </c>
       <c r="C136" s="20" t="inlineStr">
@@ -8175,7 +8175,7 @@
       </c>
       <c r="D136" s="21" t="inlineStr">
         <is>
-          <t>OSE 43 Moodle Extensión</t>
+          <t>Facultad de Derecho concurso méritos</t>
         </is>
       </c>
       <c r="E136" s="20" t="inlineStr">
@@ -8197,7 +8197,7 @@
       </c>
       <c r="B137" s="15" t="inlineStr">
         <is>
-          <t>P1991</t>
+          <t>P2066</t>
         </is>
       </c>
       <c r="C137" s="15" t="inlineStr">
@@ -8207,12 +8207,12 @@
       </c>
       <c r="D137" s="16" t="inlineStr">
         <is>
-          <t>Dinara de UNAL</t>
+          <t>OSE 26 Admisiones</t>
         </is>
       </c>
       <c r="E137" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F137" s="16" t="inlineStr">
@@ -8229,7 +8229,7 @@
       </c>
       <c r="B138" s="20" t="inlineStr">
         <is>
-          <t>P2061</t>
+          <t>P2067</t>
         </is>
       </c>
       <c r="C138" s="20" t="inlineStr">
@@ -8239,7 +8239,7 @@
       </c>
       <c r="D138" s="21" t="inlineStr">
         <is>
-          <t>Dinara de UNAL</t>
+          <t>OSE 43 Moodle Extensión</t>
         </is>
       </c>
       <c r="E138" s="20" t="inlineStr">
@@ -8261,7 +8261,7 @@
       </c>
       <c r="B139" s="15" t="inlineStr">
         <is>
-          <t>P2062</t>
+          <t>P2560</t>
         </is>
       </c>
       <c r="C139" s="15" t="inlineStr">
@@ -8271,12 +8271,12 @@
       </c>
       <c r="D139" s="16" t="inlineStr">
         <is>
-          <t>Facultad de Derecho</t>
+          <t>OSE 43 Moodle Extensión</t>
         </is>
       </c>
       <c r="E139" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F139" s="16" t="inlineStr">
@@ -8293,7 +8293,7 @@
       </c>
       <c r="B140" s="20" t="inlineStr">
         <is>
-          <t>P2556</t>
+          <t>P1991</t>
         </is>
       </c>
       <c r="C140" s="20" t="inlineStr">
@@ -8303,7 +8303,7 @@
       </c>
       <c r="D140" s="21" t="inlineStr">
         <is>
-          <t>Facultad de Derecho</t>
+          <t>Dinara de UNAL</t>
         </is>
       </c>
       <c r="E140" s="20" t="inlineStr">
@@ -8325,7 +8325,7 @@
       </c>
       <c r="B141" s="15" t="inlineStr">
         <is>
-          <t>P2065</t>
+          <t>P2061</t>
         </is>
       </c>
       <c r="C141" s="15" t="inlineStr">
@@ -8335,7 +8335,7 @@
       </c>
       <c r="D141" s="16" t="inlineStr">
         <is>
-          <t>Unisalud</t>
+          <t>Dinara de UNAL</t>
         </is>
       </c>
       <c r="E141" s="15" t="inlineStr">
@@ -8357,7 +8357,7 @@
       </c>
       <c r="B142" s="20" t="inlineStr">
         <is>
-          <t>P2059</t>
+          <t>P2062</t>
         </is>
       </c>
       <c r="C142" s="20" t="inlineStr">
@@ -8367,7 +8367,7 @@
       </c>
       <c r="D142" s="21" t="inlineStr">
         <is>
-          <t>Contrato 4 - Servicio Computacion</t>
+          <t>Facultad de Derecho</t>
         </is>
       </c>
       <c r="E142" s="20" t="inlineStr">
@@ -8389,7 +8389,7 @@
       </c>
       <c r="B143" s="15" t="inlineStr">
         <is>
-          <t>P2068</t>
+          <t>P2556</t>
         </is>
       </c>
       <c r="C143" s="15" t="inlineStr">
@@ -8399,7 +8399,7 @@
       </c>
       <c r="D143" s="16" t="inlineStr">
         <is>
-          <t>Contrato 4 - Servicio Computacion</t>
+          <t>Facultad de Derecho</t>
         </is>
       </c>
       <c r="E143" s="15" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="B144" s="20" t="inlineStr">
         <is>
-          <t>P2063</t>
+          <t>P2065</t>
         </is>
       </c>
       <c r="C144" s="20" t="inlineStr">
@@ -8431,7 +8431,7 @@
       </c>
       <c r="D144" s="21" t="inlineStr">
         <is>
-          <t>Ofc Gestion Ambiental</t>
+          <t>Unisalud</t>
         </is>
       </c>
       <c r="E144" s="20" t="inlineStr">
@@ -8453,7 +8453,7 @@
       </c>
       <c r="B145" s="15" t="inlineStr">
         <is>
-          <t>P2064</t>
+          <t>P2059</t>
         </is>
       </c>
       <c r="C145" s="15" t="inlineStr">
@@ -8463,12 +8463,12 @@
       </c>
       <c r="D145" s="16" t="inlineStr">
         <is>
-          <t>Ofc Gestion Ambiental</t>
+          <t>Contrato 4 - Servicio Computacion</t>
         </is>
       </c>
       <c r="E145" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F145" s="16" t="inlineStr">
@@ -8485,27 +8485,27 @@
       </c>
       <c r="B146" s="20" t="inlineStr">
         <is>
-          <t>P2121</t>
+          <t>P2068</t>
         </is>
       </c>
       <c r="C146" s="20" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>UNA</t>
         </is>
       </c>
       <c r="D146" s="21" t="inlineStr">
         <is>
-          <t>Agente Cognitivo e Infraestructura AWS</t>
+          <t>Contrato 4 - Servicio Computacion</t>
         </is>
       </c>
       <c r="E146" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F146" s="21" t="inlineStr">
         <is>
-          <t>Unidad Administrativa Especial de Catastro Distrital</t>
+          <t>Universidad Nacional de Colombia</t>
         </is>
       </c>
     </row>
@@ -8517,27 +8517,27 @@
       </c>
       <c r="B147" s="15" t="inlineStr">
         <is>
-          <t>P2122</t>
+          <t>P2063</t>
         </is>
       </c>
       <c r="C147" s="15" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>UNA</t>
         </is>
       </c>
       <c r="D147" s="16" t="inlineStr">
         <is>
-          <t>Agente Cognitivo e Infraestructura AWS</t>
+          <t>Ofc Gestion Ambiental</t>
         </is>
       </c>
       <c r="E147" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F147" s="16" t="inlineStr">
         <is>
-          <t>Unidad Administrativa Especial de Catastro Distrital</t>
+          <t>Universidad Nacional de Colombia</t>
         </is>
       </c>
     </row>
@@ -8549,27 +8549,27 @@
       </c>
       <c r="B148" s="20" t="inlineStr">
         <is>
-          <t>P2123</t>
+          <t>P2064</t>
         </is>
       </c>
       <c r="C148" s="20" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>UNA</t>
         </is>
       </c>
       <c r="D148" s="21" t="inlineStr">
         <is>
-          <t>Agente Cognitivo e Infraestructura AWS</t>
+          <t>Ofc Gestion Ambiental</t>
         </is>
       </c>
       <c r="E148" s="20" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F148" s="21" t="inlineStr">
         <is>
-          <t>Unidad Administrativa Especial de Catastro Distrital</t>
+          <t>Universidad Nacional de Colombia</t>
         </is>
       </c>
     </row>
@@ -8581,7 +8581,7 @@
       </c>
       <c r="B149" s="15" t="inlineStr">
         <is>
-          <t>P2124</t>
+          <t>P2121</t>
         </is>
       </c>
       <c r="C149" s="15" t="inlineStr">
@@ -8596,7 +8596,7 @@
       </c>
       <c r="E149" s="15" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F149" s="16" t="inlineStr">
@@ -8613,17 +8613,17 @@
       </c>
       <c r="B150" s="20" t="inlineStr">
         <is>
-          <t>P2214</t>
+          <t>P2122</t>
         </is>
       </c>
       <c r="C150" s="20" t="inlineStr">
         <is>
-          <t>PRO</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D150" s="21" t="inlineStr">
         <is>
-          <t>SmartCash - Operación</t>
+          <t>Agente Cognitivo e Infraestructura AWS</t>
         </is>
       </c>
       <c r="E150" s="20" t="inlineStr">
@@ -8633,7 +8633,7 @@
       </c>
       <c r="F150" s="21" t="inlineStr">
         <is>
-          <t>Progresión</t>
+          <t>Unidad Administrativa Especial de Catastro Distrital</t>
         </is>
       </c>
     </row>
@@ -8645,27 +8645,27 @@
       </c>
       <c r="B151" s="15" t="inlineStr">
         <is>
-          <t>P2215</t>
+          <t>P2123</t>
         </is>
       </c>
       <c r="C151" s="15" t="inlineStr">
         <is>
-          <t>PRO</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D151" s="16" t="inlineStr">
         <is>
-          <t>SmartCash - Operación</t>
+          <t>Agente Cognitivo e Infraestructura AWS</t>
         </is>
       </c>
       <c r="E151" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F151" s="16" t="inlineStr">
         <is>
-          <t>Progresión</t>
+          <t>Unidad Administrativa Especial de Catastro Distrital</t>
         </is>
       </c>
     </row>
@@ -8677,17 +8677,17 @@
       </c>
       <c r="B152" s="20" t="inlineStr">
         <is>
-          <t>P2243</t>
+          <t>P2124</t>
         </is>
       </c>
       <c r="C152" s="20" t="inlineStr">
         <is>
-          <t>UNA</t>
+          <t>CAT</t>
         </is>
       </c>
       <c r="D152" s="21" t="inlineStr">
         <is>
-          <t>Secretaría General</t>
+          <t>Agente Cognitivo e Infraestructura AWS</t>
         </is>
       </c>
       <c r="E152" s="20" t="inlineStr">
@@ -8697,7 +8697,7 @@
       </c>
       <c r="F152" s="21" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Colombia</t>
+          <t>Unidad Administrativa Especial de Catastro Distrital</t>
         </is>
       </c>
     </row>
@@ -8709,27 +8709,27 @@
       </c>
       <c r="B153" s="15" t="inlineStr">
         <is>
-          <t>P2246</t>
+          <t>P2214</t>
         </is>
       </c>
       <c r="C153" s="15" t="inlineStr">
         <is>
-          <t>UNA</t>
+          <t>PRO</t>
         </is>
       </c>
       <c r="D153" s="16" t="inlineStr">
         <is>
-          <t>Secretaría General</t>
+          <t>SmartCash - Operación</t>
         </is>
       </c>
       <c r="E153" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F153" s="16" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Colombia</t>
+          <t>Progresión</t>
         </is>
       </c>
     </row>
@@ -8741,17 +8741,17 @@
       </c>
       <c r="B154" s="20" t="inlineStr">
         <is>
-          <t>P2427</t>
+          <t>P2215</t>
         </is>
       </c>
       <c r="C154" s="20" t="inlineStr">
         <is>
-          <t>UNA</t>
+          <t>PRO</t>
         </is>
       </c>
       <c r="D154" s="21" t="inlineStr">
         <is>
-          <t>Egresados Cloud</t>
+          <t>SmartCash - Operación</t>
         </is>
       </c>
       <c r="E154" s="20" t="inlineStr">
@@ -8761,7 +8761,7 @@
       </c>
       <c r="F154" s="21" t="inlineStr">
         <is>
-          <t>Universidad Nacional de Colombia</t>
+          <t>Progresión</t>
         </is>
       </c>
     </row>
@@ -8773,7 +8773,7 @@
       </c>
       <c r="B155" s="15" t="inlineStr">
         <is>
-          <t>P2428</t>
+          <t>P2243</t>
         </is>
       </c>
       <c r="C155" s="15" t="inlineStr">
@@ -8783,12 +8783,12 @@
       </c>
       <c r="D155" s="16" t="inlineStr">
         <is>
-          <t>Egresados Cloud</t>
+          <t>Secretaría General</t>
         </is>
       </c>
       <c r="E155" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F155" s="16" t="inlineStr">
@@ -8805,7 +8805,7 @@
       </c>
       <c r="B156" s="20" t="inlineStr">
         <is>
-          <t>P2429</t>
+          <t>P2246</t>
         </is>
       </c>
       <c r="C156" s="20" t="inlineStr">
@@ -8815,7 +8815,7 @@
       </c>
       <c r="D156" s="21" t="inlineStr">
         <is>
-          <t>Egresados Cloud</t>
+          <t>Secretaría General</t>
         </is>
       </c>
       <c r="E156" s="20" t="inlineStr">
@@ -8837,7 +8837,7 @@
       </c>
       <c r="B157" s="15" t="inlineStr">
         <is>
-          <t>P2569</t>
+          <t>P2427</t>
         </is>
       </c>
       <c r="C157" s="15" t="inlineStr">
@@ -8847,7 +8847,7 @@
       </c>
       <c r="D157" s="16" t="inlineStr">
         <is>
-          <t>Fortinet 2</t>
+          <t>Egresados Cloud</t>
         </is>
       </c>
       <c r="E157" s="15" t="inlineStr">
@@ -8869,7 +8869,7 @@
       </c>
       <c r="B158" s="20" t="inlineStr">
         <is>
-          <t>P2570</t>
+          <t>P2428</t>
         </is>
       </c>
       <c r="C158" s="20" t="inlineStr">
@@ -8879,12 +8879,12 @@
       </c>
       <c r="D158" s="21" t="inlineStr">
         <is>
-          <t>Fortinet 2</t>
+          <t>Egresados Cloud</t>
         </is>
       </c>
       <c r="E158" s="20" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F158" s="21" t="inlineStr">
@@ -8901,7 +8901,7 @@
       </c>
       <c r="B159" s="15" t="inlineStr">
         <is>
-          <t>P2571</t>
+          <t>P2429</t>
         </is>
       </c>
       <c r="C159" s="15" t="inlineStr">
@@ -8911,12 +8911,12 @@
       </c>
       <c r="D159" s="16" t="inlineStr">
         <is>
-          <t>Fortinet 2</t>
+          <t>Egresados Cloud</t>
         </is>
       </c>
       <c r="E159" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F159" s="16" t="inlineStr">
@@ -8933,7 +8933,7 @@
       </c>
       <c r="B160" s="20" t="inlineStr">
         <is>
-          <t>P2572</t>
+          <t>P2569</t>
         </is>
       </c>
       <c r="C160" s="20" t="inlineStr">
@@ -8948,7 +8948,7 @@
       </c>
       <c r="E160" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F160" s="21" t="inlineStr">
@@ -8965,27 +8965,27 @@
       </c>
       <c r="B161" s="15" t="inlineStr">
         <is>
-          <t>P2639</t>
+          <t>P2570</t>
         </is>
       </c>
       <c r="C161" s="15" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>UNA</t>
         </is>
       </c>
       <c r="D161" s="16" t="inlineStr">
         <is>
-          <t>Quicksight Operación 2026</t>
+          <t>Fortinet 2</t>
         </is>
       </c>
       <c r="E161" s="15" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F161" s="16" t="inlineStr">
         <is>
-          <t>Fiduagraria</t>
+          <t>Universidad Nacional de Colombia</t>
         </is>
       </c>
     </row>
@@ -8997,27 +8997,27 @@
       </c>
       <c r="B162" s="20" t="inlineStr">
         <is>
-          <t>P2635</t>
+          <t>P2571</t>
         </is>
       </c>
       <c r="C162" s="20" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>UNA</t>
         </is>
       </c>
       <c r="D162" s="21" t="inlineStr">
         <is>
-          <t>CP Suite ( Smartcash) Operación 2026</t>
+          <t>Fortinet 2</t>
         </is>
       </c>
       <c r="E162" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F162" s="21" t="inlineStr">
         <is>
-          <t>Fiduagraria</t>
+          <t>Universidad Nacional de Colombia</t>
         </is>
       </c>
     </row>
@@ -9029,27 +9029,27 @@
       </c>
       <c r="B163" s="15" t="inlineStr">
         <is>
-          <t>P2636</t>
+          <t>P2572</t>
         </is>
       </c>
       <c r="C163" s="15" t="inlineStr">
         <is>
-          <t>AGR</t>
+          <t>UNA</t>
         </is>
       </c>
       <c r="D163" s="16" t="inlineStr">
         <is>
-          <t>CP Suite ( Smartcash) Operación 2026</t>
+          <t>Fortinet 2</t>
         </is>
       </c>
       <c r="E163" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F163" s="16" t="inlineStr">
         <is>
-          <t>Fiduagraria</t>
+          <t>Universidad Nacional de Colombia</t>
         </is>
       </c>
     </row>
@@ -9061,7 +9061,7 @@
       </c>
       <c r="B164" s="20" t="inlineStr">
         <is>
-          <t>P2637</t>
+          <t>P2639</t>
         </is>
       </c>
       <c r="C164" s="20" t="inlineStr">
@@ -9071,7 +9071,7 @@
       </c>
       <c r="D164" s="21" t="inlineStr">
         <is>
-          <t>CP Suite ( Smartcash) Operación 2026</t>
+          <t>Quicksight Operación 2026</t>
         </is>
       </c>
       <c r="E164" s="20" t="inlineStr">
@@ -9093,7 +9093,7 @@
       </c>
       <c r="B165" s="15" t="inlineStr">
         <is>
-          <t>P2638</t>
+          <t>P2635</t>
         </is>
       </c>
       <c r="C165" s="15" t="inlineStr">
@@ -9108,7 +9108,7 @@
       </c>
       <c r="E165" s="15" t="inlineStr">
         <is>
-          <t>Software SW</t>
+          <t>Implementación</t>
         </is>
       </c>
       <c r="F165" s="16" t="inlineStr">
@@ -9125,27 +9125,27 @@
       </c>
       <c r="B166" s="20" t="inlineStr">
         <is>
-          <t>P2736</t>
+          <t>P2636</t>
         </is>
       </c>
       <c r="C166" s="20" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="D166" s="21" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>CP Suite ( Smartcash) Operación 2026</t>
         </is>
       </c>
       <c r="E166" s="20" t="inlineStr">
         <is>
-          <t>Implementación</t>
+          <t>Operación</t>
         </is>
       </c>
       <c r="F166" s="21" t="inlineStr">
         <is>
-          <t>Catastro</t>
+          <t>Fiduagraria</t>
         </is>
       </c>
     </row>
@@ -9157,27 +9157,27 @@
       </c>
       <c r="B167" s="15" t="inlineStr">
         <is>
-          <t>P2737</t>
+          <t>P2637</t>
         </is>
       </c>
       <c r="C167" s="15" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="D167" s="16" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>CP Suite ( Smartcash) Operación 2026</t>
         </is>
       </c>
       <c r="E167" s="15" t="inlineStr">
         <is>
-          <t>Operación</t>
+          <t>Data</t>
         </is>
       </c>
       <c r="F167" s="16" t="inlineStr">
         <is>
-          <t>Catastro</t>
+          <t>Fiduagraria</t>
         </is>
       </c>
     </row>
@@ -9189,27 +9189,27 @@
       </c>
       <c r="B168" s="20" t="inlineStr">
         <is>
-          <t>P2738</t>
+          <t>P2638</t>
         </is>
       </c>
       <c r="C168" s="20" t="inlineStr">
         <is>
-          <t>CAT</t>
+          <t>AGR</t>
         </is>
       </c>
       <c r="D168" s="21" t="inlineStr">
         <is>
-          <t>Fase 3</t>
+          <t>CP Suite ( Smartcash) Operación 2026</t>
         </is>
       </c>
       <c r="E168" s="20" t="inlineStr">
         <is>
-          <t>Data</t>
+          <t>Software SW</t>
         </is>
       </c>
       <c r="F168" s="21" t="inlineStr">
         <is>
-          <t>Catatro</t>
+          <t>Fiduagraria</t>
         </is>
       </c>
     </row>
@@ -9221,25 +9221,121 @@
       </c>
       <c r="B169" s="15" t="inlineStr">
         <is>
+          <t>P2736</t>
+        </is>
+      </c>
+      <c r="C169" s="15" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="D169" s="16" t="inlineStr">
+        <is>
+          <t>Fase 3</t>
+        </is>
+      </c>
+      <c r="E169" s="15" t="inlineStr">
+        <is>
+          <t>Implementación</t>
+        </is>
+      </c>
+      <c r="F169" s="16" t="inlineStr">
+        <is>
+          <t>Catastro</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="18" customHeight="1">
+      <c r="A170" s="20" t="inlineStr">
+        <is>
+          <t>Oscar Barragan</t>
+        </is>
+      </c>
+      <c r="B170" s="20" t="inlineStr">
+        <is>
+          <t>P2737</t>
+        </is>
+      </c>
+      <c r="C170" s="20" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="D170" s="21" t="inlineStr">
+        <is>
+          <t>Fase 3</t>
+        </is>
+      </c>
+      <c r="E170" s="20" t="inlineStr">
+        <is>
+          <t>Operación</t>
+        </is>
+      </c>
+      <c r="F170" s="21" t="inlineStr">
+        <is>
+          <t>Catastro</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="18" customHeight="1">
+      <c r="A171" s="15" t="inlineStr">
+        <is>
+          <t>Oscar Barragan</t>
+        </is>
+      </c>
+      <c r="B171" s="15" t="inlineStr">
+        <is>
+          <t>P2738</t>
+        </is>
+      </c>
+      <c r="C171" s="15" t="inlineStr">
+        <is>
+          <t>CAT</t>
+        </is>
+      </c>
+      <c r="D171" s="16" t="inlineStr">
+        <is>
+          <t>Fase 3</t>
+        </is>
+      </c>
+      <c r="E171" s="15" t="inlineStr">
+        <is>
+          <t>Data</t>
+        </is>
+      </c>
+      <c r="F171" s="16" t="inlineStr">
+        <is>
+          <t>Catatro</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="A172" s="20" t="inlineStr">
+        <is>
+          <t>Oscar Barragan</t>
+        </is>
+      </c>
+      <c r="B172" s="20" t="inlineStr">
+        <is>
           <t>P2717</t>
         </is>
       </c>
-      <c r="C169" s="15" t="inlineStr">
+      <c r="C172" s="20" t="inlineStr">
         <is>
           <t>UCA</t>
         </is>
       </c>
-      <c r="D169" s="16" t="inlineStr">
+      <c r="D172" s="21" t="inlineStr">
         <is>
           <t>Renovación Semestre 1 - 2025</t>
         </is>
       </c>
-      <c r="E169" s="15" t="inlineStr">
+      <c r="E172" s="20" t="inlineStr">
         <is>
           <t>Operación</t>
         </is>
       </c>
-      <c r="F169" s="16" t="inlineStr">
+      <c r="F172" s="21" t="inlineStr">
         <is>
           <t>Universidad de Caldas</t>
         </is>

</xml_diff>